<commit_message>
Generators day by day: GN20 line 6 (1276701) never came to site; asset at GN20 to be given
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
@@ -1673,7 +1673,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1276701</t>
+          <t>to be given</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1791,7 +1791,7 @@
       </c>
       <c r="AQ11" t="inlineStr">
         <is>
-          <t>Baseplan says 365 kVA; a 350 kVA was asked for, priced at the card's 315 kVA line (no 350 line)</t>
+          <t>Baseplan line 6 is 1276701, a 365 kVA that NEVER CAME TO SITE (Andrew, 22 Oct): close that line and raise the right one for the set that is at GN20. A 350 kVA was asked for, on site 30 Sep, asset number to be given; priced at the card's 315 kVA line (no 350 line)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Generators workbook: labour and transport a set, with hire, now and later
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Day by day" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates &amp; basis" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Labour &amp; transport" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rates &amp; basis" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -65,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -74,6 +75,7 @@
     <xf numFmtId="4" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="4" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -2541,6 +2543,969 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="50" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Ref</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>kVA</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>On site</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Install (done)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Demob (at demob)</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Transport each way</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Delivery leg (done)</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Pickup leg (at demob)</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Hire standby to 22 Oct</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Hire race days</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Hire total</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Set total now (hire + install + delivery)</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Set total later (demob + pickup)</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Set total</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>GN01</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>28 Sep</t>
+        </is>
+      </c>
+      <c r="D2" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E2" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F2" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G2" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H2" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I2" s="4" t="n">
+        <v>2412.52</v>
+      </c>
+      <c r="J2" s="4" t="n">
+        <v>579</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>2991.52</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>3587.26</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>4183</v>
+      </c>
+      <c r="O2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>GN03</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>01 Oct</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H3" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I3" s="4" t="n">
+        <v>1556.88</v>
+      </c>
+      <c r="J3" s="4" t="n">
+        <v>424.6</v>
+      </c>
+      <c r="K3" s="4" t="n">
+        <v>1981.48</v>
+      </c>
+      <c r="L3" s="4" t="n">
+        <v>2427.22</v>
+      </c>
+      <c r="M3" s="4" t="n">
+        <v>445.74</v>
+      </c>
+      <c r="N3" s="4" t="n">
+        <v>2872.96</v>
+      </c>
+      <c r="O3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>GN04</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H4" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I4" s="4" t="n">
+        <v>283.07</v>
+      </c>
+      <c r="J4" s="4" t="n">
+        <v>424.6</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>707.67</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>1153.41</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>445.74</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>1599.15</v>
+      </c>
+      <c r="O4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GN06</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>15 Oct</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H5" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I5" s="4" t="n">
+        <v>729.12</v>
+      </c>
+      <c r="J5" s="4" t="n">
+        <v>546.84</v>
+      </c>
+      <c r="K5" s="4" t="n">
+        <v>1275.96</v>
+      </c>
+      <c r="L5" s="4" t="n">
+        <v>1871.7</v>
+      </c>
+      <c r="M5" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N5" s="4" t="n">
+        <v>2467.44</v>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Baseplan says 60 kVA from 19 Oct; a 50 kVA was asked for, on site 15 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>GN10</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H6" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I6" s="4" t="n">
+        <v>244.47</v>
+      </c>
+      <c r="J6" s="4" t="n">
+        <v>366.69</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>611.16</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>1056.9</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>445.74</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>1502.64</v>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>Baseplan says 60 kVA; a 20 kVA was asked for</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>GN13</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>45</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>12 Oct</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E7" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F7" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G7" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I7" s="4" t="n">
+        <v>967.15</v>
+      </c>
+      <c r="J7" s="4" t="n">
+        <v>527.52</v>
+      </c>
+      <c r="K7" s="4" t="n">
+        <v>1494.67</v>
+      </c>
+      <c r="L7" s="4" t="n">
+        <v>1940.41</v>
+      </c>
+      <c r="M7" s="4" t="n">
+        <v>445.74</v>
+      </c>
+      <c r="N7" s="4" t="n">
+        <v>2386.15</v>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>Baseplan says 60 kVA delivered as 45, term 12 Nov; a 45 kVA was asked for, hire ends 25 Oct</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>GN18</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>07 Oct</t>
+        </is>
+      </c>
+      <c r="D8" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E8" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F8" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G8" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H8" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I8" s="4" t="n">
+        <v>1458.23</v>
+      </c>
+      <c r="J8" s="4" t="n">
+        <v>546.84</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2005.07</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>2600.81</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>3196.55</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>Baseplan says 60 kVA; a 50 kVA was asked for</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>GN19</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H9" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I9" s="4" t="n">
+        <v>386</v>
+      </c>
+      <c r="J9" s="4" t="n">
+        <v>579</v>
+      </c>
+      <c r="K9" s="4" t="n">
+        <v>965</v>
+      </c>
+      <c r="L9" s="4" t="n">
+        <v>1560.74</v>
+      </c>
+      <c r="M9" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N9" s="4" t="n">
+        <v>2156.48</v>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>Baseplan says 80 kVA delivered as 60; a 60 kVA was asked for</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>GN20</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>350</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>30 Sep</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H10" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="I10" s="4" t="n">
+        <v>5425.48</v>
+      </c>
+      <c r="J10" s="4" t="n">
+        <v>1415.34</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>6840.82</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>7607.38</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>766.5599999999999</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>8373.940000000001</v>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>350 kVA: no card line for labour or transport; the 200 kVA figures are used</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>GN21</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>30 Sep</t>
+        </is>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H11" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I11" s="4" t="n">
+        <v>2219.52</v>
+      </c>
+      <c r="J11" s="4" t="n">
+        <v>579</v>
+      </c>
+      <c r="K11" s="4" t="n">
+        <v>2798.52</v>
+      </c>
+      <c r="L11" s="4" t="n">
+        <v>3394.26</v>
+      </c>
+      <c r="M11" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N11" s="4" t="n">
+        <v>3990</v>
+      </c>
+      <c r="O11" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GN23</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>150</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>30 Sep</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="E12" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="F12" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H12" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I12" s="4" t="n">
+        <v>3082.66</v>
+      </c>
+      <c r="J12" s="4" t="n">
+        <v>804.17</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>3886.83</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>4503.39</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>616.5599999999999</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>5119.95</v>
+      </c>
+      <c r="O12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>GN24</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E13" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F13" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="H13" s="4" t="n">
+        <v>450</v>
+      </c>
+      <c r="I13" s="4" t="n">
+        <v>386</v>
+      </c>
+      <c r="J13" s="4" t="n">
+        <v>579</v>
+      </c>
+      <c r="K13" s="4" t="n">
+        <v>965</v>
+      </c>
+      <c r="L13" s="4" t="n">
+        <v>1560.74</v>
+      </c>
+      <c r="M13" s="4" t="n">
+        <v>595.74</v>
+      </c>
+      <c r="N13" s="4" t="n">
+        <v>2156.48</v>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>trailer-mounted 60 kVA; not yet priced on our page (no rate or date recorded) - priced here at the 60 kVA line</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>GN25</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>19 Oct</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="E14" s="4" t="n">
+        <v>145.74</v>
+      </c>
+      <c r="F14" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="H14" s="4" t="n">
+        <v>300</v>
+      </c>
+      <c r="I14" s="4" t="n">
+        <v>244.47</v>
+      </c>
+      <c r="J14" s="4" t="n">
+        <v>366.69</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>611.16</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>1056.9</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>445.74</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>1502.64</v>
+      </c>
+      <c r="O14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>GN26</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12 Oct</t>
+        </is>
+      </c>
+      <c r="D15" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="E15" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="F15" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H15" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="I15" s="4" t="n">
+        <v>2005.07</v>
+      </c>
+      <c r="J15" s="4" t="n">
+        <v>1093.67</v>
+      </c>
+      <c r="K15" s="4" t="n">
+        <v>3098.74</v>
+      </c>
+      <c r="L15" s="4" t="n">
+        <v>3865.3</v>
+      </c>
+      <c r="M15" s="4" t="n">
+        <v>766.5599999999999</v>
+      </c>
+      <c r="N15" s="4" t="n">
+        <v>4631.86</v>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>GN27</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>200</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>12 Oct</t>
+        </is>
+      </c>
+      <c r="D16" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="E16" s="4" t="n">
+        <v>166.56</v>
+      </c>
+      <c r="F16" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="H16" s="4" t="n">
+        <v>600</v>
+      </c>
+      <c r="I16" s="4" t="n">
+        <v>2005.07</v>
+      </c>
+      <c r="J16" s="4" t="n">
+        <v>1093.67</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>3098.74</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>3865.3</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>766.5599999999999</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>4631.86</v>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="17"/>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>15 sets</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr"/>
+      <c r="D18" s="6" t="n">
+        <v>2269.38</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>2269.38</v>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="6" t="n">
+        <v>6450</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>6450</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>23405.71</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>9926.629999999999</v>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>33332.34</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>42051.72</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>8719.379999999999</v>
+      </c>
+      <c r="N18" s="6" t="n">
+        <v>50771.1</v>
+      </c>
+      <c r="O18" s="5" t="inlineStr"/>
+    </row>
+    <row r="19"/>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Baseplan 9961976 lines 51-55: labour 11 x $291.48 + 4 x $333.12 = $4,538.76 (install + demob a set, the card's figures, on 15 sets); transport 10 x $300 + 14 x $450 + 6 x $600 = $12,900 (both legs, 15 sets). Both count GN20's 1276701, which never came: labour and transport are 14 sets.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2551,22 +3516,22 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
+      <c r="A1" s="7" t="inlineStr">
         <is>
           <t>kVA</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="B1" s="7" t="inlineStr">
         <is>
           <t>Card line</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="7" t="inlineStr">
         <is>
           <t>Full daily rate 2026</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="D1" s="7" t="inlineStr">
         <is>
           <t>Standby rate 2026</t>
         </is>

</xml_diff>

<commit_message>
Generators workbook: GN20 off the list, GN24 as the 60 kVA 1277089, labour and transport a set
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GNRrrx1C9yJ5N627f7yfrr
</commit_message>
<xml_diff>
--- a/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
+++ b/03_GC500_Delivery_Control/review_22Oct2026_baseplan6_schedule13/GC500_9961976_Generators_DayByDay_22Oct2026.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ18"/>
+  <dimension ref="A1:AQ17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -1665,17 +1665,17 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GN20</t>
+          <t>GN21</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>to be given</t>
+          <t>1261284</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -1684,133 +1684,129 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>235.8906</v>
+        <v>96.50069999999999</v>
       </c>
       <c r="F11" t="n">
-        <v>471.7812</v>
+        <v>193.0014</v>
       </c>
       <c r="I11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="J11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="L11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="M11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="N11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="O11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="P11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="R11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="T11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="U11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="V11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="W11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="X11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="Y11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AA11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AB11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AC11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AD11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AE11" s="2" t="n">
-        <v>235.89</v>
+        <v>96.5</v>
       </c>
       <c r="AF11" s="3" t="n">
-        <v>471.78</v>
+        <v>193</v>
       </c>
       <c r="AG11" s="3" t="n">
-        <v>471.78</v>
+        <v>193</v>
       </c>
       <c r="AH11" s="3" t="n">
-        <v>471.78</v>
+        <v>193</v>
       </c>
       <c r="AI11" t="n">
         <v>23</v>
       </c>
       <c r="AJ11" s="4" t="n">
-        <v>5425.48</v>
+        <v>2219.52</v>
       </c>
       <c r="AK11" t="n">
         <v>3</v>
       </c>
       <c r="AL11" s="4" t="n">
-        <v>1415.34</v>
+        <v>579</v>
       </c>
       <c r="AM11" s="4" t="n">
-        <v>6840.83</v>
+        <v>2798.52</v>
       </c>
       <c r="AN11" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
       <c r="AO11" s="4" t="n">
-        <v>6260.4</v>
+        <v>868.5</v>
       </c>
       <c r="AP11" s="4" t="n">
-        <v>580.4299999999999</v>
-      </c>
-      <c r="AQ11" t="inlineStr">
-        <is>
-          <t>Baseplan line 6 is 1276701, a 365 kVA that NEVER CAME TO SITE (Andrew, 22 Oct): close that line and raise the right one for the set that is at GN20. A 350 kVA was asked for, on site 30 Sep, asset number to be given; priced at the card's 315 kVA line (no 350 line)</t>
-        </is>
-      </c>
+        <v>1930.02</v>
+      </c>
+      <c r="AQ11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GN21</t>
+          <t>GN23</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>150</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>1261284</t>
+          <t>1297157</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1819,260 +1815,207 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>96.50069999999999</v>
+        <v>134.0288</v>
       </c>
       <c r="F12" t="n">
-        <v>193.0014</v>
+        <v>268.0575</v>
       </c>
       <c r="I12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="J12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="L12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="M12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="N12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="O12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="P12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="Q12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="R12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="T12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="U12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="V12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="W12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="X12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="Y12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AA12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AB12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AD12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AE12" s="2" t="n">
-        <v>96.5</v>
+        <v>134.03</v>
       </c>
       <c r="AF12" s="3" t="n">
-        <v>193</v>
+        <v>268.06</v>
       </c>
       <c r="AG12" s="3" t="n">
-        <v>193</v>
+        <v>268.06</v>
       </c>
       <c r="AH12" s="3" t="n">
-        <v>193</v>
+        <v>268.06</v>
       </c>
       <c r="AI12" t="n">
         <v>23</v>
       </c>
       <c r="AJ12" s="4" t="n">
-        <v>2219.52</v>
+        <v>3082.66</v>
       </c>
       <c r="AK12" t="n">
         <v>3</v>
       </c>
       <c r="AL12" s="4" t="n">
-        <v>579</v>
+        <v>804.17</v>
       </c>
       <c r="AM12" s="4" t="n">
-        <v>2798.52</v>
+        <v>3886.83</v>
       </c>
       <c r="AN12" t="n">
-        <v>38</v>
+        <v>9</v>
       </c>
       <c r="AO12" s="4" t="n">
-        <v>868.5</v>
+        <v>2412.54</v>
       </c>
       <c r="AP12" s="4" t="n">
-        <v>1930.02</v>
+        <v>1474.29</v>
       </c>
       <c r="AQ12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GN23</t>
+          <t>GN24</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>1297157</t>
+          <t>1277089</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>30 Sep</t>
+          <t>19 Oct</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>134.0288</v>
+        <v>96.50069999999999</v>
       </c>
       <c r="F13" t="n">
-        <v>268.0575</v>
-      </c>
-      <c r="I13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="J13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="K13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="L13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="M13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="N13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="O13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="P13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="Q13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="R13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="S13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="T13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="U13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="V13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="W13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="X13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="Y13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="Z13" s="2" t="n">
-        <v>134.03</v>
-      </c>
-      <c r="AA13" s="2" t="n">
-        <v>134.03</v>
+        <v>193.0014</v>
       </c>
       <c r="AB13" s="2" t="n">
-        <v>134.03</v>
+        <v>96.5</v>
       </c>
       <c r="AC13" s="2" t="n">
-        <v>134.03</v>
+        <v>96.5</v>
       </c>
       <c r="AD13" s="2" t="n">
-        <v>134.03</v>
+        <v>96.5</v>
       </c>
       <c r="AE13" s="2" t="n">
-        <v>134.03</v>
+        <v>96.5</v>
       </c>
       <c r="AF13" s="3" t="n">
-        <v>268.06</v>
+        <v>193</v>
       </c>
       <c r="AG13" s="3" t="n">
-        <v>268.06</v>
+        <v>193</v>
       </c>
       <c r="AH13" s="3" t="n">
-        <v>268.06</v>
+        <v>193</v>
       </c>
       <c r="AI13" t="n">
-        <v>23</v>
+        <v>4</v>
       </c>
       <c r="AJ13" s="4" t="n">
-        <v>3082.66</v>
+        <v>386</v>
       </c>
       <c r="AK13" t="n">
         <v>3</v>
       </c>
       <c r="AL13" s="4" t="n">
-        <v>804.17</v>
+        <v>579</v>
       </c>
       <c r="AM13" s="4" t="n">
-        <v>3886.83</v>
+        <v>965.01</v>
       </c>
       <c r="AN13" t="n">
-        <v>9</v>
+        <v>49</v>
       </c>
       <c r="AO13" s="4" t="n">
-        <v>2412.54</v>
+        <v>984.33</v>
       </c>
       <c r="AP13" s="4" t="n">
-        <v>1474.29</v>
-      </c>
-      <c r="AQ13" t="inlineStr"/>
+        <v>-19.32</v>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>Andrew, 22 Oct: charged as a 60 kVA, asset 1277089, on site 19 Oct. Baseplan (6) has line 49 Off Rent at $0 and line 17 (1276412, the 80 kVA) gone: line 49 needs to be on rent from 19 Oct at the 60 kVA rate</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GN24</t>
+          <t>GN25</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>1277089</t>
+          <t>1244536</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2081,140 +2024,161 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>96.50069999999999</v>
+        <v>61.1171</v>
       </c>
       <c r="F14" t="n">
-        <v>193.0014</v>
+        <v>122.2301</v>
       </c>
       <c r="AB14" s="2" t="n">
-        <v>96.5</v>
+        <v>61.12</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>96.5</v>
+        <v>61.12</v>
       </c>
       <c r="AD14" s="2" t="n">
-        <v>96.5</v>
+        <v>61.12</v>
       </c>
       <c r="AE14" s="2" t="n">
-        <v>96.5</v>
+        <v>61.12</v>
       </c>
       <c r="AF14" s="3" t="n">
-        <v>193</v>
+        <v>122.23</v>
       </c>
       <c r="AG14" s="3" t="n">
-        <v>193</v>
+        <v>122.23</v>
       </c>
       <c r="AH14" s="3" t="n">
-        <v>193</v>
+        <v>122.23</v>
       </c>
       <c r="AI14" t="n">
         <v>4</v>
       </c>
       <c r="AJ14" s="4" t="n">
-        <v>386</v>
+        <v>244.47</v>
       </c>
       <c r="AK14" t="n">
         <v>3</v>
       </c>
       <c r="AL14" s="4" t="n">
-        <v>579</v>
+        <v>366.69</v>
       </c>
       <c r="AM14" s="4" t="n">
-        <v>965.01</v>
+        <v>611.16</v>
       </c>
       <c r="AN14" t="n">
-        <v>49</v>
+        <v>18</v>
       </c>
       <c r="AO14" s="4" t="n">
-        <v>984.33</v>
+        <v>855.63</v>
       </c>
       <c r="AP14" s="4" t="n">
-        <v>-19.32</v>
-      </c>
-      <c r="AQ14" t="inlineStr">
-        <is>
-          <t>trailer-mounted 60 kVA; not yet priced on our page (no rate or date recorded) - priced here at the 60 kVA line</t>
-        </is>
-      </c>
+        <v>-244.47</v>
+      </c>
+      <c r="AQ14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GN25</t>
+          <t>GN26</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>1244536</t>
+          <t>1316182</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>19 Oct</t>
+          <t>12 Oct</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>61.1171</v>
+        <v>182.2791</v>
       </c>
       <c r="F15" t="n">
-        <v>122.2301</v>
+        <v>364.5582</v>
+      </c>
+      <c r="U15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="V15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="W15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="X15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="Y15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="Z15" s="2" t="n">
+        <v>182.28</v>
+      </c>
+      <c r="AA15" s="2" t="n">
+        <v>182.28</v>
       </c>
       <c r="AB15" s="2" t="n">
-        <v>61.12</v>
+        <v>182.28</v>
       </c>
       <c r="AC15" s="2" t="n">
-        <v>61.12</v>
+        <v>182.28</v>
       </c>
       <c r="AD15" s="2" t="n">
-        <v>61.12</v>
+        <v>182.28</v>
       </c>
       <c r="AE15" s="2" t="n">
-        <v>61.12</v>
+        <v>182.28</v>
       </c>
       <c r="AF15" s="3" t="n">
-        <v>122.23</v>
+        <v>364.56</v>
       </c>
       <c r="AG15" s="3" t="n">
-        <v>122.23</v>
+        <v>364.56</v>
       </c>
       <c r="AH15" s="3" t="n">
-        <v>122.23</v>
+        <v>364.56</v>
       </c>
       <c r="AI15" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="AJ15" s="4" t="n">
-        <v>244.47</v>
+        <v>2005.07</v>
       </c>
       <c r="AK15" t="n">
         <v>3</v>
       </c>
       <c r="AL15" s="4" t="n">
-        <v>366.69</v>
+        <v>1093.67</v>
       </c>
       <c r="AM15" s="4" t="n">
-        <v>611.16</v>
+        <v>3098.74</v>
       </c>
       <c r="AN15" t="n">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="AO15" s="4" t="n">
-        <v>855.63</v>
+        <v>2005.08</v>
       </c>
       <c r="AP15" s="4" t="n">
-        <v>-244.47</v>
-      </c>
-      <c r="AQ15" t="inlineStr"/>
+        <v>1093.66</v>
+      </c>
+      <c r="AQ15" t="inlineStr">
+        <is>
+          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>GN26</t>
+          <t>GN27</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -2224,7 +2188,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>1316182</t>
+          <t>1316183</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2296,239 +2260,140 @@
         <v>3098.74</v>
       </c>
       <c r="AN16" t="n">
+        <v>43</v>
+      </c>
+      <c r="AO16" s="4" t="n">
+        <v>2551.92</v>
+      </c>
+      <c r="AP16" s="4" t="n">
+        <v>546.8200000000001</v>
+      </c>
+      <c r="AQ16" t="inlineStr">
+        <is>
+          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr"/>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="5" t="inlineStr"/>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="5" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>96.5</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>327.03</v>
+      </c>
+      <c r="J17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="K17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="L17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="M17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="N17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="O17" s="5" t="n">
+        <v>397.8</v>
+      </c>
+      <c r="P17" s="5" t="n">
+        <v>488.94</v>
+      </c>
+      <c r="Q17" s="5" t="n">
+        <v>488.94</v>
+      </c>
+      <c r="R17" s="5" t="n">
+        <v>488.94</v>
+      </c>
+      <c r="S17" s="5" t="n">
+        <v>488.94</v>
+      </c>
+      <c r="T17" s="5" t="n">
+        <v>488.94</v>
+      </c>
+      <c r="U17" s="5" t="n">
+        <v>941.42</v>
+      </c>
+      <c r="V17" s="5" t="n">
+        <v>941.42</v>
+      </c>
+      <c r="W17" s="5" t="n">
+        <v>941.42</v>
+      </c>
+      <c r="X17" s="5" t="n">
+        <v>1032.56</v>
+      </c>
+      <c r="Y17" s="5" t="n">
+        <v>1032.56</v>
+      </c>
+      <c r="Z17" s="5" t="n">
+        <v>1032.56</v>
+      </c>
+      <c r="AA17" s="5" t="n">
+        <v>1032.56</v>
+      </c>
+      <c r="AB17" s="5" t="n">
+        <v>1418.56</v>
+      </c>
+      <c r="AC17" s="5" t="n">
+        <v>1418.56</v>
+      </c>
+      <c r="AD17" s="5" t="n">
+        <v>1418.56</v>
+      </c>
+      <c r="AE17" s="5" t="n">
+        <v>1418.56</v>
+      </c>
+      <c r="AF17" s="5" t="n">
+        <v>2837.1</v>
+      </c>
+      <c r="AG17" s="5" t="n">
+        <v>2837.1</v>
+      </c>
+      <c r="AH17" s="5" t="n">
+        <v>2837.1</v>
+      </c>
+      <c r="AI17" s="5" t="n">
+        <v>170</v>
+      </c>
+      <c r="AJ17" s="5" t="n">
+        <v>17980.22</v>
+      </c>
+      <c r="AK17" s="5" t="n">
         <v>42</v>
       </c>
-      <c r="AO16" s="4" t="n">
-        <v>2005.08</v>
-      </c>
-      <c r="AP16" s="4" t="n">
-        <v>1093.66</v>
-      </c>
-      <c r="AQ16" t="inlineStr">
-        <is>
-          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>GN27</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>1316183</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>12 Oct</t>
-        </is>
-      </c>
-      <c r="E17" t="n">
-        <v>182.2791</v>
-      </c>
-      <c r="F17" t="n">
-        <v>364.5582</v>
-      </c>
-      <c r="U17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="V17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="W17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="X17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="Y17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="Z17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AA17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AB17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AC17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AD17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AE17" s="2" t="n">
-        <v>182.28</v>
-      </c>
-      <c r="AF17" s="3" t="n">
-        <v>364.56</v>
-      </c>
-      <c r="AG17" s="3" t="n">
-        <v>364.56</v>
-      </c>
-      <c r="AH17" s="3" t="n">
-        <v>364.56</v>
-      </c>
-      <c r="AI17" t="n">
-        <v>11</v>
-      </c>
-      <c r="AJ17" s="4" t="n">
-        <v>2005.07</v>
-      </c>
-      <c r="AK17" t="n">
-        <v>3</v>
-      </c>
-      <c r="AL17" s="4" t="n">
-        <v>1093.67</v>
-      </c>
-      <c r="AM17" s="4" t="n">
-        <v>3098.74</v>
-      </c>
-      <c r="AN17" t="n">
-        <v>43</v>
-      </c>
-      <c r="AO17" s="4" t="n">
-        <v>2551.92</v>
-      </c>
-      <c r="AP17" s="4" t="n">
-        <v>546.8200000000001</v>
-      </c>
-      <c r="AQ17" t="inlineStr">
-        <is>
-          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B18" s="5" t="inlineStr"/>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="5" t="inlineStr"/>
-      <c r="E18" s="5" t="inlineStr"/>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="5" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="H18" s="5" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="I18" s="5" t="n">
-        <v>562.92</v>
-      </c>
-      <c r="J18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="L18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="N18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="O18" s="5" t="n">
-        <v>633.6900000000001</v>
-      </c>
-      <c r="P18" s="5" t="n">
-        <v>724.83</v>
-      </c>
-      <c r="Q18" s="5" t="n">
-        <v>724.83</v>
-      </c>
-      <c r="R18" s="5" t="n">
-        <v>724.83</v>
-      </c>
-      <c r="S18" s="5" t="n">
-        <v>724.83</v>
-      </c>
-      <c r="T18" s="5" t="n">
-        <v>724.83</v>
-      </c>
-      <c r="U18" s="5" t="n">
-        <v>1177.31</v>
-      </c>
-      <c r="V18" s="5" t="n">
-        <v>1177.31</v>
-      </c>
-      <c r="W18" s="5" t="n">
-        <v>1177.31</v>
-      </c>
-      <c r="X18" s="5" t="n">
-        <v>1268.45</v>
-      </c>
-      <c r="Y18" s="5" t="n">
-        <v>1268.45</v>
-      </c>
-      <c r="Z18" s="5" t="n">
-        <v>1268.45</v>
-      </c>
-      <c r="AA18" s="5" t="n">
-        <v>1268.45</v>
-      </c>
-      <c r="AB18" s="5" t="n">
-        <v>1654.45</v>
-      </c>
-      <c r="AC18" s="5" t="n">
-        <v>1654.45</v>
-      </c>
-      <c r="AD18" s="5" t="n">
-        <v>1654.45</v>
-      </c>
-      <c r="AE18" s="5" t="n">
-        <v>1654.45</v>
-      </c>
-      <c r="AF18" s="5" t="n">
-        <v>3308.89</v>
-      </c>
-      <c r="AG18" s="5" t="n">
-        <v>3308.89</v>
-      </c>
-      <c r="AH18" s="5" t="n">
-        <v>3308.89</v>
-      </c>
-      <c r="AI18" s="5" t="n">
-        <v>193</v>
-      </c>
-      <c r="AJ18" s="5" t="n">
-        <v>23405.71</v>
-      </c>
-      <c r="AK18" s="5" t="n">
-        <v>45</v>
-      </c>
-      <c r="AL18" s="5" t="n">
-        <v>9926.66</v>
-      </c>
-      <c r="AM18" s="5" t="n">
-        <v>33332.36</v>
-      </c>
-      <c r="AN18" s="5" t="inlineStr"/>
-      <c r="AO18" s="5" t="n">
-        <v>26711.01</v>
-      </c>
-      <c r="AP18" s="5" t="n">
-        <v>6621.35</v>
-      </c>
-      <c r="AQ18" s="5" t="inlineStr">
-        <is>
-          <t>15 sets</t>
+      <c r="AL17" s="5" t="n">
+        <v>8511.309999999999</v>
+      </c>
+      <c r="AM17" s="5" t="n">
+        <v>26491.54</v>
+      </c>
+      <c r="AN17" s="5" t="inlineStr"/>
+      <c r="AO17" s="5" t="n">
+        <v>20450.61</v>
+      </c>
+      <c r="AP17" s="5" t="n">
+        <v>6040.93</v>
+      </c>
+      <c r="AQ17" s="5" t="inlineStr">
+        <is>
+          <t>14 sets</t>
         </is>
       </c>
     </row>
@@ -2543,7 +2408,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O20"/>
+  <dimension ref="A1:O19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -3071,12 +2936,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>GN20</t>
+          <t>GN21</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>350</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -3085,53 +2950,49 @@
         </is>
       </c>
       <c r="D10" s="4" t="n">
-        <v>166.56</v>
+        <v>145.74</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>166.56</v>
+        <v>145.74</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>600</v>
+        <v>450</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>5425.48</v>
+        <v>2219.52</v>
       </c>
       <c r="J10" s="4" t="n">
-        <v>1415.34</v>
+        <v>579</v>
       </c>
       <c r="K10" s="4" t="n">
-        <v>6840.82</v>
+        <v>2798.52</v>
       </c>
       <c r="L10" s="4" t="n">
-        <v>7607.38</v>
+        <v>3394.26</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>766.5599999999999</v>
+        <v>595.74</v>
       </c>
       <c r="N10" s="4" t="n">
-        <v>8373.940000000001</v>
-      </c>
-      <c r="O10" t="inlineStr">
-        <is>
-          <t>350 kVA: no card line for labour or transport; the 200 kVA figures are used</t>
-        </is>
-      </c>
+        <v>3990</v>
+      </c>
+      <c r="O10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GN21</t>
+          <t>GN23</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>150</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -3140,10 +3001,10 @@
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>145.74</v>
+        <v>166.56</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>145.74</v>
+        <v>166.56</v>
       </c>
       <c r="F11" s="4" t="n">
         <v>450</v>
@@ -3155,46 +3016,46 @@
         <v>450</v>
       </c>
       <c r="I11" s="4" t="n">
-        <v>2219.52</v>
+        <v>3082.66</v>
       </c>
       <c r="J11" s="4" t="n">
-        <v>579</v>
+        <v>804.17</v>
       </c>
       <c r="K11" s="4" t="n">
-        <v>2798.52</v>
+        <v>3886.83</v>
       </c>
       <c r="L11" s="4" t="n">
-        <v>3394.26</v>
+        <v>4503.39</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>595.74</v>
+        <v>616.5599999999999</v>
       </c>
       <c r="N11" s="4" t="n">
-        <v>3990</v>
+        <v>5119.95</v>
       </c>
       <c r="O11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>GN23</t>
+          <t>GN24</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>150</t>
+          <t>60</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>30 Sep</t>
+          <t>19 Oct</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>166.56</v>
+        <v>145.74</v>
       </c>
       <c r="E12" s="4" t="n">
-        <v>166.56</v>
+        <v>145.74</v>
       </c>
       <c r="F12" s="4" t="n">
         <v>450</v>
@@ -3206,34 +3067,38 @@
         <v>450</v>
       </c>
       <c r="I12" s="4" t="n">
-        <v>3082.66</v>
+        <v>386</v>
       </c>
       <c r="J12" s="4" t="n">
-        <v>804.17</v>
+        <v>579</v>
       </c>
       <c r="K12" s="4" t="n">
-        <v>3886.83</v>
+        <v>965</v>
       </c>
       <c r="L12" s="4" t="n">
-        <v>4503.39</v>
+        <v>1560.74</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>616.5599999999999</v>
+        <v>595.74</v>
       </c>
       <c r="N12" s="4" t="n">
-        <v>5119.95</v>
-      </c>
-      <c r="O12" t="inlineStr"/>
+        <v>2156.48</v>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>Andrew, 22 Oct: charged as a 60 kVA, asset 1277089, on site 19 Oct. Baseplan (6) has line 49 Off Rent at $0 and line 17 (1276412, the 80 kVA) gone: line 49 needs to be on rent from 19 Oct at the 60 kVA rate</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GN24</t>
+          <t>GN25</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>60</t>
+          <t>20</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -3248,93 +3113,93 @@
         <v>145.74</v>
       </c>
       <c r="F13" s="4" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>450</v>
+        <v>300</v>
       </c>
       <c r="I13" s="4" t="n">
-        <v>386</v>
+        <v>244.47</v>
       </c>
       <c r="J13" s="4" t="n">
-        <v>579</v>
+        <v>366.69</v>
       </c>
       <c r="K13" s="4" t="n">
-        <v>965</v>
+        <v>611.16</v>
       </c>
       <c r="L13" s="4" t="n">
-        <v>1560.74</v>
+        <v>1056.9</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>595.74</v>
+        <v>445.74</v>
       </c>
       <c r="N13" s="4" t="n">
-        <v>2156.48</v>
-      </c>
-      <c r="O13" t="inlineStr">
-        <is>
-          <t>trailer-mounted 60 kVA; not yet priced on our page (no rate or date recorded) - priced here at the 60 kVA line</t>
-        </is>
-      </c>
+        <v>1502.64</v>
+      </c>
+      <c r="O13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GN25</t>
+          <t>GN26</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>20</t>
+          <t>200</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>19 Oct</t>
+          <t>12 Oct</t>
         </is>
       </c>
       <c r="D14" s="4" t="n">
-        <v>145.74</v>
+        <v>166.56</v>
       </c>
       <c r="E14" s="4" t="n">
-        <v>145.74</v>
+        <v>166.56</v>
       </c>
       <c r="F14" s="4" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>300</v>
+        <v>600</v>
       </c>
       <c r="I14" s="4" t="n">
-        <v>244.47</v>
+        <v>2005.07</v>
       </c>
       <c r="J14" s="4" t="n">
-        <v>366.69</v>
+        <v>1093.67</v>
       </c>
       <c r="K14" s="4" t="n">
-        <v>611.16</v>
+        <v>3098.74</v>
       </c>
       <c r="L14" s="4" t="n">
-        <v>1056.9</v>
+        <v>3865.3</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>445.74</v>
+        <v>766.5599999999999</v>
       </c>
       <c r="N14" s="4" t="n">
-        <v>1502.64</v>
-      </c>
-      <c r="O14" t="inlineStr"/>
+        <v>4631.86</v>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GN26</t>
+          <t>GN27</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -3386,112 +3251,57 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>GN27</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>200</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>12 Oct</t>
-        </is>
-      </c>
-      <c r="D16" s="4" t="n">
-        <v>166.56</v>
-      </c>
-      <c r="E16" s="4" t="n">
-        <v>166.56</v>
-      </c>
-      <c r="F16" s="4" t="n">
-        <v>600</v>
-      </c>
-      <c r="G16" s="4" t="n">
-        <v>600</v>
-      </c>
-      <c r="H16" s="4" t="n">
-        <v>600</v>
-      </c>
-      <c r="I16" s="4" t="n">
-        <v>2005.07</v>
-      </c>
-      <c r="J16" s="4" t="n">
-        <v>1093.67</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>3098.74</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>3865.3</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>766.5599999999999</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>4631.86</v>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>concert set; on our page only as "GN?" - to be given its own reference</t>
-        </is>
-      </c>
-    </row>
-    <row r="17"/>
-    <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="5" t="inlineStr">
-        <is>
-          <t>15 sets</t>
-        </is>
-      </c>
-      <c r="C18" s="5" t="inlineStr"/>
-      <c r="D18" s="6" t="n">
-        <v>2269.38</v>
-      </c>
-      <c r="E18" s="6" t="n">
-        <v>2269.38</v>
-      </c>
-      <c r="F18" s="5" t="inlineStr"/>
-      <c r="G18" s="6" t="n">
-        <v>6450</v>
-      </c>
-      <c r="H18" s="6" t="n">
-        <v>6450</v>
-      </c>
-      <c r="I18" s="6" t="n">
-        <v>23405.71</v>
-      </c>
-      <c r="J18" s="6" t="n">
-        <v>9926.629999999999</v>
-      </c>
-      <c r="K18" s="6" t="n">
-        <v>33332.34</v>
-      </c>
-      <c r="L18" s="6" t="n">
-        <v>42051.72</v>
-      </c>
-      <c r="M18" s="6" t="n">
-        <v>8719.379999999999</v>
-      </c>
-      <c r="N18" s="6" t="n">
-        <v>50771.1</v>
-      </c>
-      <c r="O18" s="5" t="inlineStr"/>
-    </row>
-    <row r="19"/>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Baseplan 9961976 lines 51-55: labour 11 x $291.48 + 4 x $333.12 = $4,538.76 (install + demob a set, the card's figures, on 15 sets); transport 10 x $300 + 14 x $450 + 6 x $600 = $12,900 (both legs, 15 sets). Both count GN20's 1276701, which never came: labour and transport are 14 sets.</t>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>14 sets</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr"/>
+      <c r="D17" s="6" t="n">
+        <v>2102.82</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>2102.82</v>
+      </c>
+      <c r="F17" s="5" t="inlineStr"/>
+      <c r="G17" s="6" t="n">
+        <v>5850</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>5850</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>17980.23</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>8511.290000000001</v>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>26491.52</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>34444.34</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>7952.82</v>
+      </c>
+      <c r="N17" s="6" t="n">
+        <v>42397.16</v>
+      </c>
+      <c r="O17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18"/>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Baseplan 9961976 lines 51-55: labour 11 x $291.48 + 4 x $333.12 = $4,538.76 (install + demob a set, the card's figures, on 15 sets); transport 10 x $300 + 14 x $450 + 6 x $600 = $12,900 (both legs, 15 sets). The record has 14 sets (GN20 is off the list on Andrew's word, 22 Oct: 1276701 never came): labour is 10 x $291.48 + 3 x $333.12 = $3,914.16 and transport 10 x $300 + 14 x $450 + 4 x $600 = $11,700, and Baseplan charges demob and the pickup leg before the work.</t>
         </is>
       </c>
     </row>
@@ -3506,7 +3316,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -3663,26 +3473,8 @@
         <v>182.2791</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>350</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Generator 315 KVA (next size down; no 350 line)</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>471.7812</v>
-      </c>
-      <c r="D9" t="n">
-        <v>235.8906</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
+    <row r="10">
+      <c r="A10" t="inlineStr">
         <is>
           <t>Basis: the 2026 street card, ex GST. Standby rate every day from the day the set lands until 22 Oct; full daily rate on the race days 23, 24 and 25 Oct; no hire charge after 25 Oct. The rate follows the size the customer asked for, not the size sent. On-site dates are the site record. Author: Andrew Fisher, 22 Oct 2026.</t>
         </is>

</xml_diff>